<commit_message>
fix: update .gitignore to include coverage files; refactor PrintTeamEliminationMatches for clarity
</commit_message>
<xml_diff>
--- a/pools-example-large.xlsx
+++ b/pools-example-large.xlsx
@@ -7098,7 +7098,7 @@
         <f>data!$B$3</f>
       </c>
       <c r="I19" s="21" t="str">
-        <f>data!$B$8</f>
+        <f>data!$B$6</f>
       </c>
       <c r="J19" s="21"/>
       <c r="K19" s="21"/>
@@ -7106,7 +7106,7 @@
       <c r="M19" s="21"/>
       <c r="N19" s="21"/>
       <c r="O19" s="21" t="str">
-        <f>data!$B$7</f>
+        <f>data!$B$8</f>
       </c>
     </row>
     <row r="20">
@@ -7250,7 +7250,7 @@
         <f>data!$B$3</f>
       </c>
       <c r="I26" s="21" t="str">
-        <f>data!$B$8</f>
+        <f>data!$B$6</f>
       </c>
       <c r="J26" s="21" t="s">
         <v>239</v>
@@ -7266,7 +7266,7 @@
         <v>239</v>
       </c>
       <c r="O26" s="21" t="str">
-        <f>data!$B$7</f>
+        <f>data!$B$8</f>
       </c>
     </row>
     <row r="27">
@@ -7334,7 +7334,7 @@
         <f>data!$B$5</f>
       </c>
       <c r="I32" s="21" t="str">
-        <f>data!$B$8</f>
+        <f>data!$B$7</f>
       </c>
       <c r="J32" s="21"/>
       <c r="K32" s="21"/>
@@ -7342,7 +7342,7 @@
       <c r="M32" s="21"/>
       <c r="N32" s="21"/>
       <c r="O32" s="21" t="str">
-        <f>data!$B$6</f>
+        <f>data!$B$8</f>
       </c>
     </row>
     <row r="33">
@@ -7486,7 +7486,7 @@
         <f>data!$B$5</f>
       </c>
       <c r="I39" s="21" t="str">
-        <f>data!$B$8</f>
+        <f>data!$B$7</f>
       </c>
       <c r="J39" s="21" t="s">
         <v>239</v>
@@ -7502,7 +7502,7 @@
         <v>239</v>
       </c>
       <c r="O39" s="21" t="str">
-        <f>data!$B$6</f>
+        <f>data!$B$8</f>
       </c>
     </row>
     <row r="40">
@@ -7982,7 +7982,7 @@
     </row>
     <row r="76">
       <c r="A76" s="21" t="str">
-        <f>data!$B$11</f>
+        <f>data!$B$9</f>
       </c>
       <c r="B76" s="21"/>
       <c r="C76" s="21"/>
@@ -7990,10 +7990,10 @@
       <c r="E76" s="21"/>
       <c r="F76" s="21"/>
       <c r="G76" s="21" t="str">
-        <f>data!$B$10</f>
+        <f>data!$B$11</f>
       </c>
       <c r="I76" s="21" t="str">
-        <f>data!$B$14</f>
+        <f>data!$B$12</f>
       </c>
       <c r="J76" s="21"/>
       <c r="K76" s="21"/>
@@ -8001,7 +8001,7 @@
       <c r="M76" s="21"/>
       <c r="N76" s="21"/>
       <c r="O76" s="21" t="str">
-        <f>data!$B$13</f>
+        <f>data!$B$14</f>
       </c>
     </row>
     <row r="77">
@@ -8126,7 +8126,7 @@
     </row>
     <row r="83">
       <c r="A83" s="21" t="str">
-        <f>data!$B$11</f>
+        <f>data!$B$9</f>
       </c>
       <c r="B83" s="21" t="s">
         <v>239</v>
@@ -8142,10 +8142,10 @@
         <v>239</v>
       </c>
       <c r="G83" s="21" t="str">
-        <f>data!$B$10</f>
+        <f>data!$B$11</f>
       </c>
       <c r="I83" s="21" t="str">
-        <f>data!$B$14</f>
+        <f>data!$B$12</f>
       </c>
       <c r="J83" s="21" t="s">
         <v>239</v>
@@ -8161,7 +8161,7 @@
         <v>239</v>
       </c>
       <c r="O83" s="21" t="str">
-        <f>data!$B$13</f>
+        <f>data!$B$14</f>
       </c>
     </row>
     <row r="84">
@@ -8218,7 +8218,7 @@
     </row>
     <row r="89">
       <c r="A89" s="21" t="str">
-        <f>data!$B$11</f>
+        <f>data!$B$10</f>
       </c>
       <c r="B89" s="21"/>
       <c r="C89" s="21"/>
@@ -8226,10 +8226,10 @@
       <c r="E89" s="21"/>
       <c r="F89" s="21"/>
       <c r="G89" s="21" t="str">
-        <f>data!$B$9</f>
+        <f>data!$B$11</f>
       </c>
       <c r="I89" s="21" t="str">
-        <f>data!$B$14</f>
+        <f>data!$B$13</f>
       </c>
       <c r="J89" s="21"/>
       <c r="K89" s="21"/>
@@ -8237,7 +8237,7 @@
       <c r="M89" s="21"/>
       <c r="N89" s="21"/>
       <c r="O89" s="21" t="str">
-        <f>data!$B$12</f>
+        <f>data!$B$14</f>
       </c>
     </row>
     <row r="90">
@@ -8362,7 +8362,7 @@
     </row>
     <row r="96">
       <c r="A96" s="21" t="str">
-        <f>data!$B$11</f>
+        <f>data!$B$10</f>
       </c>
       <c r="B96" s="21" t="s">
         <v>239</v>
@@ -8378,10 +8378,10 @@
         <v>239</v>
       </c>
       <c r="G96" s="21" t="str">
-        <f>data!$B$9</f>
+        <f>data!$B$11</f>
       </c>
       <c r="I96" s="21" t="str">
-        <f>data!$B$14</f>
+        <f>data!$B$13</f>
       </c>
       <c r="J96" s="21" t="s">
         <v>239</v>
@@ -8397,7 +8397,7 @@
         <v>239</v>
       </c>
       <c r="O96" s="21" t="str">
-        <f>data!$B$12</f>
+        <f>data!$B$14</f>
       </c>
     </row>
     <row r="97">
@@ -8740,7 +8740,7 @@
     </row>
     <row r="119">
       <c r="A119" s="21" t="str">
-        <f>data!$B$17</f>
+        <f>data!$B$15</f>
       </c>
       <c r="B119" s="21"/>
       <c r="C119" s="21"/>
@@ -8748,10 +8748,10 @@
       <c r="E119" s="21"/>
       <c r="F119" s="21"/>
       <c r="G119" s="21" t="str">
-        <f>data!$B$16</f>
+        <f>data!$B$17</f>
       </c>
       <c r="I119" s="21" t="str">
-        <f>data!$B$20</f>
+        <f>data!$B$18</f>
       </c>
       <c r="J119" s="21"/>
       <c r="K119" s="21"/>
@@ -8759,7 +8759,7 @@
       <c r="M119" s="21"/>
       <c r="N119" s="21"/>
       <c r="O119" s="21" t="str">
-        <f>data!$B$19</f>
+        <f>data!$B$20</f>
       </c>
     </row>
     <row r="120">
@@ -8884,7 +8884,7 @@
     </row>
     <row r="126">
       <c r="A126" s="21" t="str">
-        <f>data!$B$17</f>
+        <f>data!$B$15</f>
       </c>
       <c r="B126" s="21" t="s">
         <v>239</v>
@@ -8900,10 +8900,10 @@
         <v>239</v>
       </c>
       <c r="G126" s="21" t="str">
-        <f>data!$B$16</f>
+        <f>data!$B$17</f>
       </c>
       <c r="I126" s="21" t="str">
-        <f>data!$B$20</f>
+        <f>data!$B$18</f>
       </c>
       <c r="J126" s="21" t="s">
         <v>239</v>
@@ -8919,7 +8919,7 @@
         <v>239</v>
       </c>
       <c r="O126" s="21" t="str">
-        <f>data!$B$19</f>
+        <f>data!$B$20</f>
       </c>
     </row>
     <row r="127">
@@ -8976,7 +8976,7 @@
     </row>
     <row r="132">
       <c r="A132" s="21" t="str">
-        <f>data!$B$17</f>
+        <f>data!$B$16</f>
       </c>
       <c r="B132" s="21"/>
       <c r="C132" s="21"/>
@@ -8984,10 +8984,10 @@
       <c r="E132" s="21"/>
       <c r="F132" s="21"/>
       <c r="G132" s="21" t="str">
-        <f>data!$B$15</f>
+        <f>data!$B$17</f>
       </c>
       <c r="I132" s="21" t="str">
-        <f>data!$B$20</f>
+        <f>data!$B$19</f>
       </c>
       <c r="J132" s="21"/>
       <c r="K132" s="21"/>
@@ -8995,7 +8995,7 @@
       <c r="M132" s="21"/>
       <c r="N132" s="21"/>
       <c r="O132" s="21" t="str">
-        <f>data!$B$18</f>
+        <f>data!$B$20</f>
       </c>
     </row>
     <row r="133">
@@ -9120,7 +9120,7 @@
     </row>
     <row r="139">
       <c r="A139" s="21" t="str">
-        <f>data!$B$17</f>
+        <f>data!$B$16</f>
       </c>
       <c r="B139" s="21" t="s">
         <v>239</v>
@@ -9136,10 +9136,10 @@
         <v>239</v>
       </c>
       <c r="G139" s="21" t="str">
-        <f>data!$B$15</f>
+        <f>data!$B$17</f>
       </c>
       <c r="I139" s="21" t="str">
-        <f>data!$B$20</f>
+        <f>data!$B$19</f>
       </c>
       <c r="J139" s="21" t="s">
         <v>239</v>
@@ -9155,7 +9155,7 @@
         <v>239</v>
       </c>
       <c r="O139" s="21" t="str">
-        <f>data!$B$18</f>
+        <f>data!$B$20</f>
       </c>
     </row>
     <row r="140">
@@ -9498,7 +9498,7 @@
     </row>
     <row r="162">
       <c r="A162" s="21" t="str">
-        <f>data!$B$23</f>
+        <f>data!$B$21</f>
       </c>
       <c r="B162" s="21"/>
       <c r="C162" s="21"/>
@@ -9506,10 +9506,10 @@
       <c r="E162" s="21"/>
       <c r="F162" s="21"/>
       <c r="G162" s="21" t="str">
-        <f>data!$B$22</f>
+        <f>data!$B$23</f>
       </c>
       <c r="I162" s="21" t="str">
-        <f>data!$B$26</f>
+        <f>data!$B$24</f>
       </c>
       <c r="J162" s="21"/>
       <c r="K162" s="21"/>
@@ -9517,7 +9517,7 @@
       <c r="M162" s="21"/>
       <c r="N162" s="21"/>
       <c r="O162" s="21" t="str">
-        <f>data!$B$25</f>
+        <f>data!$B$26</f>
       </c>
     </row>
     <row r="163">
@@ -9642,7 +9642,7 @@
     </row>
     <row r="169">
       <c r="A169" s="21" t="str">
-        <f>data!$B$23</f>
+        <f>data!$B$21</f>
       </c>
       <c r="B169" s="21" t="s">
         <v>239</v>
@@ -9658,10 +9658,10 @@
         <v>239</v>
       </c>
       <c r="G169" s="21" t="str">
-        <f>data!$B$22</f>
+        <f>data!$B$23</f>
       </c>
       <c r="I169" s="21" t="str">
-        <f>data!$B$26</f>
+        <f>data!$B$24</f>
       </c>
       <c r="J169" s="21" t="s">
         <v>239</v>
@@ -9677,7 +9677,7 @@
         <v>239</v>
       </c>
       <c r="O169" s="21" t="str">
-        <f>data!$B$25</f>
+        <f>data!$B$26</f>
       </c>
     </row>
     <row r="170">
@@ -9734,7 +9734,7 @@
     </row>
     <row r="175">
       <c r="A175" s="21" t="str">
-        <f>data!$B$23</f>
+        <f>data!$B$22</f>
       </c>
       <c r="B175" s="21"/>
       <c r="C175" s="21"/>
@@ -9742,10 +9742,10 @@
       <c r="E175" s="21"/>
       <c r="F175" s="21"/>
       <c r="G175" s="21" t="str">
-        <f>data!$B$21</f>
+        <f>data!$B$23</f>
       </c>
       <c r="I175" s="21" t="str">
-        <f>data!$B$26</f>
+        <f>data!$B$25</f>
       </c>
       <c r="J175" s="21"/>
       <c r="K175" s="21"/>
@@ -9753,7 +9753,7 @@
       <c r="M175" s="21"/>
       <c r="N175" s="21"/>
       <c r="O175" s="21" t="str">
-        <f>data!$B$24</f>
+        <f>data!$B$26</f>
       </c>
     </row>
     <row r="176">
@@ -9878,7 +9878,7 @@
     </row>
     <row r="182">
       <c r="A182" s="21" t="str">
-        <f>data!$B$23</f>
+        <f>data!$B$22</f>
       </c>
       <c r="B182" s="21" t="s">
         <v>239</v>
@@ -9894,10 +9894,10 @@
         <v>239</v>
       </c>
       <c r="G182" s="21" t="str">
-        <f>data!$B$21</f>
+        <f>data!$B$23</f>
       </c>
       <c r="I182" s="21" t="str">
-        <f>data!$B$26</f>
+        <f>data!$B$25</f>
       </c>
       <c r="J182" s="21" t="s">
         <v>239</v>
@@ -9913,7 +9913,7 @@
         <v>239</v>
       </c>
       <c r="O182" s="21" t="str">
-        <f>data!$B$24</f>
+        <f>data!$B$26</f>
       </c>
     </row>
     <row r="183">
@@ -10256,7 +10256,7 @@
     </row>
     <row r="205">
       <c r="A205" s="21" t="str">
-        <f>data!$B$29</f>
+        <f>data!$B$27</f>
       </c>
       <c r="B205" s="21"/>
       <c r="C205" s="21"/>
@@ -10264,10 +10264,10 @@
       <c r="E205" s="21"/>
       <c r="F205" s="21"/>
       <c r="G205" s="21" t="str">
-        <f>data!$B$28</f>
+        <f>data!$B$29</f>
       </c>
       <c r="I205" s="21" t="str">
-        <f>data!$B$32</f>
+        <f>data!$B$30</f>
       </c>
       <c r="J205" s="21"/>
       <c r="K205" s="21"/>
@@ -10275,7 +10275,7 @@
       <c r="M205" s="21"/>
       <c r="N205" s="21"/>
       <c r="O205" s="21" t="str">
-        <f>data!$B$31</f>
+        <f>data!$B$32</f>
       </c>
     </row>
     <row r="206">
@@ -10400,7 +10400,7 @@
     </row>
     <row r="212">
       <c r="A212" s="21" t="str">
-        <f>data!$B$29</f>
+        <f>data!$B$27</f>
       </c>
       <c r="B212" s="21" t="s">
         <v>239</v>
@@ -10416,10 +10416,10 @@
         <v>239</v>
       </c>
       <c r="G212" s="21" t="str">
-        <f>data!$B$28</f>
+        <f>data!$B$29</f>
       </c>
       <c r="I212" s="21" t="str">
-        <f>data!$B$32</f>
+        <f>data!$B$30</f>
       </c>
       <c r="J212" s="21" t="s">
         <v>239</v>
@@ -10435,7 +10435,7 @@
         <v>239</v>
       </c>
       <c r="O212" s="21" t="str">
-        <f>data!$B$31</f>
+        <f>data!$B$32</f>
       </c>
     </row>
     <row r="213">
@@ -10492,7 +10492,7 @@
     </row>
     <row r="218">
       <c r="A218" s="21" t="str">
-        <f>data!$B$29</f>
+        <f>data!$B$28</f>
       </c>
       <c r="B218" s="21"/>
       <c r="C218" s="21"/>
@@ -10500,10 +10500,10 @@
       <c r="E218" s="21"/>
       <c r="F218" s="21"/>
       <c r="G218" s="21" t="str">
-        <f>data!$B$27</f>
+        <f>data!$B$29</f>
       </c>
       <c r="I218" s="21" t="str">
-        <f>data!$B$32</f>
+        <f>data!$B$31</f>
       </c>
       <c r="J218" s="21"/>
       <c r="K218" s="21"/>
@@ -10511,7 +10511,7 @@
       <c r="M218" s="21"/>
       <c r="N218" s="21"/>
       <c r="O218" s="21" t="str">
-        <f>data!$B$30</f>
+        <f>data!$B$32</f>
       </c>
     </row>
     <row r="219">
@@ -10636,7 +10636,7 @@
     </row>
     <row r="225">
       <c r="A225" s="21" t="str">
-        <f>data!$B$29</f>
+        <f>data!$B$28</f>
       </c>
       <c r="B225" s="21" t="s">
         <v>239</v>
@@ -10652,10 +10652,10 @@
         <v>239</v>
       </c>
       <c r="G225" s="21" t="str">
-        <f>data!$B$27</f>
+        <f>data!$B$29</f>
       </c>
       <c r="I225" s="21" t="str">
-        <f>data!$B$32</f>
+        <f>data!$B$31</f>
       </c>
       <c r="J225" s="21" t="s">
         <v>239</v>
@@ -10671,7 +10671,7 @@
         <v>239</v>
       </c>
       <c r="O225" s="21" t="str">
-        <f>data!$B$30</f>
+        <f>data!$B$32</f>
       </c>
     </row>
     <row r="226">
@@ -11014,7 +11014,7 @@
     </row>
     <row r="248">
       <c r="A248" s="21" t="str">
-        <f>data!$B$35</f>
+        <f>data!$B$33</f>
       </c>
       <c r="B248" s="21"/>
       <c r="C248" s="21"/>
@@ -11022,10 +11022,10 @@
       <c r="E248" s="21"/>
       <c r="F248" s="21"/>
       <c r="G248" s="21" t="str">
-        <f>data!$B$34</f>
+        <f>data!$B$35</f>
       </c>
       <c r="I248" s="21" t="str">
-        <f>data!$B$38</f>
+        <f>data!$B$36</f>
       </c>
       <c r="J248" s="21"/>
       <c r="K248" s="21"/>
@@ -11033,7 +11033,7 @@
       <c r="M248" s="21"/>
       <c r="N248" s="21"/>
       <c r="O248" s="21" t="str">
-        <f>data!$B$37</f>
+        <f>data!$B$38</f>
       </c>
     </row>
     <row r="249">
@@ -11158,7 +11158,7 @@
     </row>
     <row r="255">
       <c r="A255" s="21" t="str">
-        <f>data!$B$35</f>
+        <f>data!$B$33</f>
       </c>
       <c r="B255" s="21" t="s">
         <v>239</v>
@@ -11174,10 +11174,10 @@
         <v>239</v>
       </c>
       <c r="G255" s="21" t="str">
-        <f>data!$B$34</f>
+        <f>data!$B$35</f>
       </c>
       <c r="I255" s="21" t="str">
-        <f>data!$B$38</f>
+        <f>data!$B$36</f>
       </c>
       <c r="J255" s="21" t="s">
         <v>239</v>
@@ -11193,7 +11193,7 @@
         <v>239</v>
       </c>
       <c r="O255" s="21" t="str">
-        <f>data!$B$37</f>
+        <f>data!$B$38</f>
       </c>
     </row>
     <row r="256">
@@ -11250,7 +11250,7 @@
     </row>
     <row r="261">
       <c r="A261" s="21" t="str">
-        <f>data!$B$35</f>
+        <f>data!$B$34</f>
       </c>
       <c r="B261" s="21"/>
       <c r="C261" s="21"/>
@@ -11258,10 +11258,10 @@
       <c r="E261" s="21"/>
       <c r="F261" s="21"/>
       <c r="G261" s="21" t="str">
-        <f>data!$B$33</f>
+        <f>data!$B$35</f>
       </c>
       <c r="I261" s="21" t="str">
-        <f>data!$B$38</f>
+        <f>data!$B$37</f>
       </c>
       <c r="J261" s="21"/>
       <c r="K261" s="21"/>
@@ -11269,7 +11269,7 @@
       <c r="M261" s="21"/>
       <c r="N261" s="21"/>
       <c r="O261" s="21" t="str">
-        <f>data!$B$36</f>
+        <f>data!$B$38</f>
       </c>
     </row>
     <row r="262">
@@ -11394,7 +11394,7 @@
     </row>
     <row r="268">
       <c r="A268" s="21" t="str">
-        <f>data!$B$35</f>
+        <f>data!$B$34</f>
       </c>
       <c r="B268" s="21" t="s">
         <v>239</v>
@@ -11410,10 +11410,10 @@
         <v>239</v>
       </c>
       <c r="G268" s="21" t="str">
-        <f>data!$B$33</f>
+        <f>data!$B$35</f>
       </c>
       <c r="I268" s="21" t="str">
-        <f>data!$B$38</f>
+        <f>data!$B$37</f>
       </c>
       <c r="J268" s="21" t="s">
         <v>239</v>
@@ -11429,7 +11429,7 @@
         <v>239</v>
       </c>
       <c r="O268" s="21" t="str">
-        <f>data!$B$36</f>
+        <f>data!$B$38</f>
       </c>
     </row>
     <row r="269">
@@ -11772,7 +11772,7 @@
     </row>
     <row r="291">
       <c r="A291" s="21" t="str">
-        <f>data!$B$41</f>
+        <f>data!$B$39</f>
       </c>
       <c r="B291" s="21"/>
       <c r="C291" s="21"/>
@@ -11780,10 +11780,10 @@
       <c r="E291" s="21"/>
       <c r="F291" s="21"/>
       <c r="G291" s="21" t="str">
-        <f>data!$B$40</f>
+        <f>data!$B$41</f>
       </c>
       <c r="I291" s="21" t="str">
-        <f>data!$B$44</f>
+        <f>data!$B$42</f>
       </c>
       <c r="J291" s="21"/>
       <c r="K291" s="21"/>
@@ -11791,7 +11791,7 @@
       <c r="M291" s="21"/>
       <c r="N291" s="21"/>
       <c r="O291" s="21" t="str">
-        <f>data!$B$43</f>
+        <f>data!$B$44</f>
       </c>
     </row>
     <row r="292">
@@ -11916,7 +11916,7 @@
     </row>
     <row r="298">
       <c r="A298" s="21" t="str">
-        <f>data!$B$41</f>
+        <f>data!$B$39</f>
       </c>
       <c r="B298" s="21" t="s">
         <v>239</v>
@@ -11932,10 +11932,10 @@
         <v>239</v>
       </c>
       <c r="G298" s="21" t="str">
-        <f>data!$B$40</f>
+        <f>data!$B$41</f>
       </c>
       <c r="I298" s="21" t="str">
-        <f>data!$B$44</f>
+        <f>data!$B$42</f>
       </c>
       <c r="J298" s="21" t="s">
         <v>239</v>
@@ -11951,7 +11951,7 @@
         <v>239</v>
       </c>
       <c r="O298" s="21" t="str">
-        <f>data!$B$43</f>
+        <f>data!$B$44</f>
       </c>
     </row>
     <row r="299">
@@ -12008,7 +12008,7 @@
     </row>
     <row r="304">
       <c r="A304" s="21" t="str">
-        <f>data!$B$41</f>
+        <f>data!$B$40</f>
       </c>
       <c r="B304" s="21"/>
       <c r="C304" s="21"/>
@@ -12016,10 +12016,10 @@
       <c r="E304" s="21"/>
       <c r="F304" s="21"/>
       <c r="G304" s="21" t="str">
-        <f>data!$B$39</f>
+        <f>data!$B$41</f>
       </c>
       <c r="I304" s="21" t="str">
-        <f>data!$B$44</f>
+        <f>data!$B$43</f>
       </c>
       <c r="J304" s="21"/>
       <c r="K304" s="21"/>
@@ -12027,7 +12027,7 @@
       <c r="M304" s="21"/>
       <c r="N304" s="21"/>
       <c r="O304" s="21" t="str">
-        <f>data!$B$42</f>
+        <f>data!$B$44</f>
       </c>
     </row>
     <row r="305">
@@ -12152,7 +12152,7 @@
     </row>
     <row r="311">
       <c r="A311" s="21" t="str">
-        <f>data!$B$41</f>
+        <f>data!$B$40</f>
       </c>
       <c r="B311" s="21" t="s">
         <v>239</v>
@@ -12168,10 +12168,10 @@
         <v>239</v>
       </c>
       <c r="G311" s="21" t="str">
-        <f>data!$B$39</f>
+        <f>data!$B$41</f>
       </c>
       <c r="I311" s="21" t="str">
-        <f>data!$B$44</f>
+        <f>data!$B$43</f>
       </c>
       <c r="J311" s="21" t="s">
         <v>239</v>
@@ -12187,7 +12187,7 @@
         <v>239</v>
       </c>
       <c r="O311" s="21" t="str">
-        <f>data!$B$42</f>
+        <f>data!$B$44</f>
       </c>
     </row>
     <row r="312">
@@ -12530,7 +12530,7 @@
     </row>
     <row r="334">
       <c r="A334" s="21" t="str">
-        <f>data!$B$47</f>
+        <f>data!$B$45</f>
       </c>
       <c r="B334" s="21"/>
       <c r="C334" s="21"/>
@@ -12538,10 +12538,10 @@
       <c r="E334" s="21"/>
       <c r="F334" s="21"/>
       <c r="G334" s="21" t="str">
-        <f>data!$B$46</f>
+        <f>data!$B$47</f>
       </c>
       <c r="I334" s="21" t="str">
-        <f>data!$B$50</f>
+        <f>data!$B$48</f>
       </c>
       <c r="J334" s="21"/>
       <c r="K334" s="21"/>
@@ -12549,7 +12549,7 @@
       <c r="M334" s="21"/>
       <c r="N334" s="21"/>
       <c r="O334" s="21" t="str">
-        <f>data!$B$49</f>
+        <f>data!$B$50</f>
       </c>
     </row>
     <row r="335">
@@ -12674,7 +12674,7 @@
     </row>
     <row r="341">
       <c r="A341" s="21" t="str">
-        <f>data!$B$47</f>
+        <f>data!$B$45</f>
       </c>
       <c r="B341" s="21" t="s">
         <v>239</v>
@@ -12690,10 +12690,10 @@
         <v>239</v>
       </c>
       <c r="G341" s="21" t="str">
-        <f>data!$B$46</f>
+        <f>data!$B$47</f>
       </c>
       <c r="I341" s="21" t="str">
-        <f>data!$B$50</f>
+        <f>data!$B$48</f>
       </c>
       <c r="J341" s="21" t="s">
         <v>239</v>
@@ -12709,7 +12709,7 @@
         <v>239</v>
       </c>
       <c r="O341" s="21" t="str">
-        <f>data!$B$49</f>
+        <f>data!$B$50</f>
       </c>
     </row>
     <row r="342">
@@ -12766,7 +12766,7 @@
     </row>
     <row r="347">
       <c r="A347" s="21" t="str">
-        <f>data!$B$47</f>
+        <f>data!$B$46</f>
       </c>
       <c r="B347" s="21"/>
       <c r="C347" s="21"/>
@@ -12774,10 +12774,10 @@
       <c r="E347" s="21"/>
       <c r="F347" s="21"/>
       <c r="G347" s="21" t="str">
-        <f>data!$B$45</f>
+        <f>data!$B$47</f>
       </c>
       <c r="I347" s="21" t="str">
-        <f>data!$B$50</f>
+        <f>data!$B$49</f>
       </c>
       <c r="J347" s="21"/>
       <c r="K347" s="21"/>
@@ -12785,7 +12785,7 @@
       <c r="M347" s="21"/>
       <c r="N347" s="21"/>
       <c r="O347" s="21" t="str">
-        <f>data!$B$48</f>
+        <f>data!$B$50</f>
       </c>
     </row>
     <row r="348">
@@ -12910,7 +12910,7 @@
     </row>
     <row r="354">
       <c r="A354" s="21" t="str">
-        <f>data!$B$47</f>
+        <f>data!$B$46</f>
       </c>
       <c r="B354" s="21" t="s">
         <v>239</v>
@@ -12926,10 +12926,10 @@
         <v>239</v>
       </c>
       <c r="G354" s="21" t="str">
-        <f>data!$B$45</f>
+        <f>data!$B$47</f>
       </c>
       <c r="I354" s="21" t="str">
-        <f>data!$B$50</f>
+        <f>data!$B$49</f>
       </c>
       <c r="J354" s="21" t="s">
         <v>239</v>
@@ -12945,7 +12945,7 @@
         <v>239</v>
       </c>
       <c r="O354" s="21" t="str">
-        <f>data!$B$48</f>
+        <f>data!$B$50</f>
       </c>
     </row>
     <row r="355">
@@ -13288,7 +13288,7 @@
     </row>
     <row r="377">
       <c r="A377" s="21" t="str">
-        <f>data!$B$53</f>
+        <f>data!$B$51</f>
       </c>
       <c r="B377" s="21"/>
       <c r="C377" s="21"/>
@@ -13296,10 +13296,10 @@
       <c r="E377" s="21"/>
       <c r="F377" s="21"/>
       <c r="G377" s="21" t="str">
-        <f>data!$B$52</f>
+        <f>data!$B$53</f>
       </c>
       <c r="I377" s="21" t="str">
-        <f>data!$B$56</f>
+        <f>data!$B$54</f>
       </c>
       <c r="J377" s="21"/>
       <c r="K377" s="21"/>
@@ -13307,7 +13307,7 @@
       <c r="M377" s="21"/>
       <c r="N377" s="21"/>
       <c r="O377" s="21" t="str">
-        <f>data!$B$55</f>
+        <f>data!$B$56</f>
       </c>
     </row>
     <row r="378">
@@ -13432,7 +13432,7 @@
     </row>
     <row r="384">
       <c r="A384" s="21" t="str">
-        <f>data!$B$53</f>
+        <f>data!$B$51</f>
       </c>
       <c r="B384" s="21" t="s">
         <v>239</v>
@@ -13448,10 +13448,10 @@
         <v>239</v>
       </c>
       <c r="G384" s="21" t="str">
-        <f>data!$B$52</f>
+        <f>data!$B$53</f>
       </c>
       <c r="I384" s="21" t="str">
-        <f>data!$B$56</f>
+        <f>data!$B$54</f>
       </c>
       <c r="J384" s="21" t="s">
         <v>239</v>
@@ -13467,7 +13467,7 @@
         <v>239</v>
       </c>
       <c r="O384" s="21" t="str">
-        <f>data!$B$55</f>
+        <f>data!$B$56</f>
       </c>
     </row>
     <row r="385">
@@ -13524,7 +13524,7 @@
     </row>
     <row r="390">
       <c r="A390" s="21" t="str">
-        <f>data!$B$53</f>
+        <f>data!$B$52</f>
       </c>
       <c r="B390" s="21"/>
       <c r="C390" s="21"/>
@@ -13532,10 +13532,10 @@
       <c r="E390" s="21"/>
       <c r="F390" s="21"/>
       <c r="G390" s="21" t="str">
-        <f>data!$B$51</f>
+        <f>data!$B$53</f>
       </c>
       <c r="I390" s="21" t="str">
-        <f>data!$B$56</f>
+        <f>data!$B$55</f>
       </c>
       <c r="J390" s="21"/>
       <c r="K390" s="21"/>
@@ -13543,7 +13543,7 @@
       <c r="M390" s="21"/>
       <c r="N390" s="21"/>
       <c r="O390" s="21" t="str">
-        <f>data!$B$54</f>
+        <f>data!$B$56</f>
       </c>
     </row>
     <row r="391">
@@ -13668,7 +13668,7 @@
     </row>
     <row r="397">
       <c r="A397" s="21" t="str">
-        <f>data!$B$53</f>
+        <f>data!$B$52</f>
       </c>
       <c r="B397" s="21" t="s">
         <v>239</v>
@@ -13684,10 +13684,10 @@
         <v>239</v>
       </c>
       <c r="G397" s="21" t="str">
-        <f>data!$B$51</f>
+        <f>data!$B$53</f>
       </c>
       <c r="I397" s="21" t="str">
-        <f>data!$B$56</f>
+        <f>data!$B$55</f>
       </c>
       <c r="J397" s="21" t="s">
         <v>239</v>
@@ -13703,7 +13703,7 @@
         <v>239</v>
       </c>
       <c r="O397" s="21" t="str">
-        <f>data!$B$54</f>
+        <f>data!$B$56</f>
       </c>
     </row>
     <row r="398">
@@ -14046,7 +14046,7 @@
     </row>
     <row r="420">
       <c r="A420" s="21" t="str">
-        <f>data!$B$59</f>
+        <f>data!$B$57</f>
       </c>
       <c r="B420" s="21"/>
       <c r="C420" s="21"/>
@@ -14054,10 +14054,10 @@
       <c r="E420" s="21"/>
       <c r="F420" s="21"/>
       <c r="G420" s="21" t="str">
-        <f>data!$B$58</f>
+        <f>data!$B$59</f>
       </c>
       <c r="I420" s="21" t="str">
-        <f>data!$B$62</f>
+        <f>data!$B$60</f>
       </c>
       <c r="J420" s="21"/>
       <c r="K420" s="21"/>
@@ -14065,7 +14065,7 @@
       <c r="M420" s="21"/>
       <c r="N420" s="21"/>
       <c r="O420" s="21" t="str">
-        <f>data!$B$61</f>
+        <f>data!$B$62</f>
       </c>
     </row>
     <row r="421">
@@ -14190,7 +14190,7 @@
     </row>
     <row r="427">
       <c r="A427" s="21" t="str">
-        <f>data!$B$59</f>
+        <f>data!$B$57</f>
       </c>
       <c r="B427" s="21" t="s">
         <v>239</v>
@@ -14206,10 +14206,10 @@
         <v>239</v>
       </c>
       <c r="G427" s="21" t="str">
-        <f>data!$B$58</f>
+        <f>data!$B$59</f>
       </c>
       <c r="I427" s="21" t="str">
-        <f>data!$B$62</f>
+        <f>data!$B$60</f>
       </c>
       <c r="J427" s="21" t="s">
         <v>239</v>
@@ -14225,7 +14225,7 @@
         <v>239</v>
       </c>
       <c r="O427" s="21" t="str">
-        <f>data!$B$61</f>
+        <f>data!$B$62</f>
       </c>
     </row>
     <row r="428">
@@ -14282,7 +14282,7 @@
     </row>
     <row r="433">
       <c r="A433" s="21" t="str">
-        <f>data!$B$59</f>
+        <f>data!$B$58</f>
       </c>
       <c r="B433" s="21"/>
       <c r="C433" s="21"/>
@@ -14290,10 +14290,10 @@
       <c r="E433" s="21"/>
       <c r="F433" s="21"/>
       <c r="G433" s="21" t="str">
-        <f>data!$B$57</f>
+        <f>data!$B$59</f>
       </c>
       <c r="I433" s="21" t="str">
-        <f>data!$B$62</f>
+        <f>data!$B$61</f>
       </c>
       <c r="J433" s="21"/>
       <c r="K433" s="21"/>
@@ -14301,7 +14301,7 @@
       <c r="M433" s="21"/>
       <c r="N433" s="21"/>
       <c r="O433" s="21" t="str">
-        <f>data!$B$60</f>
+        <f>data!$B$62</f>
       </c>
     </row>
     <row r="434">
@@ -14426,7 +14426,7 @@
     </row>
     <row r="440">
       <c r="A440" s="21" t="str">
-        <f>data!$B$59</f>
+        <f>data!$B$58</f>
       </c>
       <c r="B440" s="21" t="s">
         <v>239</v>
@@ -14442,10 +14442,10 @@
         <v>239</v>
       </c>
       <c r="G440" s="21" t="str">
-        <f>data!$B$57</f>
+        <f>data!$B$59</f>
       </c>
       <c r="I440" s="21" t="str">
-        <f>data!$B$62</f>
+        <f>data!$B$61</f>
       </c>
       <c r="J440" s="21" t="s">
         <v>239</v>
@@ -14461,7 +14461,7 @@
         <v>239</v>
       </c>
       <c r="O440" s="21" t="str">
-        <f>data!$B$60</f>
+        <f>data!$B$62</f>
       </c>
     </row>
     <row r="441">
@@ -14804,7 +14804,7 @@
     </row>
     <row r="463">
       <c r="A463" s="21" t="str">
-        <f>data!$B$65</f>
+        <f>data!$B$63</f>
       </c>
       <c r="B463" s="21"/>
       <c r="C463" s="21"/>
@@ -14812,10 +14812,10 @@
       <c r="E463" s="21"/>
       <c r="F463" s="21"/>
       <c r="G463" s="21" t="str">
-        <f>data!$B$64</f>
+        <f>data!$B$65</f>
       </c>
       <c r="I463" s="21" t="str">
-        <f>data!$B$68</f>
+        <f>data!$B$66</f>
       </c>
       <c r="J463" s="21"/>
       <c r="K463" s="21"/>
@@ -14823,7 +14823,7 @@
       <c r="M463" s="21"/>
       <c r="N463" s="21"/>
       <c r="O463" s="21" t="str">
-        <f>data!$B$67</f>
+        <f>data!$B$68</f>
       </c>
     </row>
     <row r="464">
@@ -14948,7 +14948,7 @@
     </row>
     <row r="470">
       <c r="A470" s="21" t="str">
-        <f>data!$B$65</f>
+        <f>data!$B$63</f>
       </c>
       <c r="B470" s="21" t="s">
         <v>239</v>
@@ -14964,10 +14964,10 @@
         <v>239</v>
       </c>
       <c r="G470" s="21" t="str">
-        <f>data!$B$64</f>
+        <f>data!$B$65</f>
       </c>
       <c r="I470" s="21" t="str">
-        <f>data!$B$68</f>
+        <f>data!$B$66</f>
       </c>
       <c r="J470" s="21" t="s">
         <v>239</v>
@@ -14983,7 +14983,7 @@
         <v>239</v>
       </c>
       <c r="O470" s="21" t="str">
-        <f>data!$B$67</f>
+        <f>data!$B$68</f>
       </c>
     </row>
     <row r="471">
@@ -15040,7 +15040,7 @@
     </row>
     <row r="476">
       <c r="A476" s="21" t="str">
-        <f>data!$B$65</f>
+        <f>data!$B$64</f>
       </c>
       <c r="B476" s="21"/>
       <c r="C476" s="21"/>
@@ -15048,10 +15048,10 @@
       <c r="E476" s="21"/>
       <c r="F476" s="21"/>
       <c r="G476" s="21" t="str">
-        <f>data!$B$63</f>
+        <f>data!$B$65</f>
       </c>
       <c r="I476" s="21" t="str">
-        <f>data!$B$68</f>
+        <f>data!$B$67</f>
       </c>
       <c r="J476" s="21"/>
       <c r="K476" s="21"/>
@@ -15059,7 +15059,7 @@
       <c r="M476" s="21"/>
       <c r="N476" s="21"/>
       <c r="O476" s="21" t="str">
-        <f>data!$B$66</f>
+        <f>data!$B$68</f>
       </c>
     </row>
     <row r="477">
@@ -15184,7 +15184,7 @@
     </row>
     <row r="483">
       <c r="A483" s="21" t="str">
-        <f>data!$B$65</f>
+        <f>data!$B$64</f>
       </c>
       <c r="B483" s="21" t="s">
         <v>239</v>
@@ -15200,10 +15200,10 @@
         <v>239</v>
       </c>
       <c r="G483" s="21" t="str">
-        <f>data!$B$63</f>
+        <f>data!$B$65</f>
       </c>
       <c r="I483" s="21" t="str">
-        <f>data!$B$68</f>
+        <f>data!$B$67</f>
       </c>
       <c r="J483" s="21" t="s">
         <v>239</v>
@@ -15219,7 +15219,7 @@
         <v>239</v>
       </c>
       <c r="O483" s="21" t="str">
-        <f>data!$B$66</f>
+        <f>data!$B$68</f>
       </c>
     </row>
     <row r="484">
@@ -15562,7 +15562,7 @@
     </row>
     <row r="506">
       <c r="A506" s="21" t="str">
-        <f>data!$B$71</f>
+        <f>data!$B$69</f>
       </c>
       <c r="B506" s="21"/>
       <c r="C506" s="21"/>
@@ -15570,10 +15570,10 @@
       <c r="E506" s="21"/>
       <c r="F506" s="21"/>
       <c r="G506" s="21" t="str">
-        <f>data!$B$70</f>
+        <f>data!$B$71</f>
       </c>
       <c r="I506" s="21" t="str">
-        <f>data!$B$74</f>
+        <f>data!$B$72</f>
       </c>
       <c r="J506" s="21"/>
       <c r="K506" s="21"/>
@@ -15581,7 +15581,7 @@
       <c r="M506" s="21"/>
       <c r="N506" s="21"/>
       <c r="O506" s="21" t="str">
-        <f>data!$B$73</f>
+        <f>data!$B$74</f>
       </c>
     </row>
     <row r="507">
@@ -15706,7 +15706,7 @@
     </row>
     <row r="513">
       <c r="A513" s="21" t="str">
-        <f>data!$B$71</f>
+        <f>data!$B$69</f>
       </c>
       <c r="B513" s="21" t="s">
         <v>239</v>
@@ -15722,10 +15722,10 @@
         <v>239</v>
       </c>
       <c r="G513" s="21" t="str">
-        <f>data!$B$70</f>
+        <f>data!$B$71</f>
       </c>
       <c r="I513" s="21" t="str">
-        <f>data!$B$74</f>
+        <f>data!$B$72</f>
       </c>
       <c r="J513" s="21" t="s">
         <v>239</v>
@@ -15741,7 +15741,7 @@
         <v>239</v>
       </c>
       <c r="O513" s="21" t="str">
-        <f>data!$B$73</f>
+        <f>data!$B$74</f>
       </c>
     </row>
     <row r="514">
@@ -15798,7 +15798,7 @@
     </row>
     <row r="519">
       <c r="A519" s="21" t="str">
-        <f>data!$B$71</f>
+        <f>data!$B$70</f>
       </c>
       <c r="B519" s="21"/>
       <c r="C519" s="21"/>
@@ -15806,10 +15806,10 @@
       <c r="E519" s="21"/>
       <c r="F519" s="21"/>
       <c r="G519" s="21" t="str">
-        <f>data!$B$69</f>
+        <f>data!$B$71</f>
       </c>
       <c r="I519" s="21" t="str">
-        <f>data!$B$74</f>
+        <f>data!$B$73</f>
       </c>
       <c r="J519" s="21"/>
       <c r="K519" s="21"/>
@@ -15817,7 +15817,7 @@
       <c r="M519" s="21"/>
       <c r="N519" s="21"/>
       <c r="O519" s="21" t="str">
-        <f>data!$B$72</f>
+        <f>data!$B$74</f>
       </c>
     </row>
     <row r="520">
@@ -15942,7 +15942,7 @@
     </row>
     <row r="526">
       <c r="A526" s="21" t="str">
-        <f>data!$B$71</f>
+        <f>data!$B$70</f>
       </c>
       <c r="B526" s="21" t="s">
         <v>239</v>
@@ -15958,10 +15958,10 @@
         <v>239</v>
       </c>
       <c r="G526" s="21" t="str">
-        <f>data!$B$69</f>
+        <f>data!$B$71</f>
       </c>
       <c r="I526" s="21" t="str">
-        <f>data!$B$74</f>
+        <f>data!$B$73</f>
       </c>
       <c r="J526" s="21" t="s">
         <v>239</v>
@@ -15977,7 +15977,7 @@
         <v>239</v>
       </c>
       <c r="O526" s="21" t="str">
-        <f>data!$B$72</f>
+        <f>data!$B$74</f>
       </c>
     </row>
     <row r="527">
@@ -16320,7 +16320,7 @@
     </row>
     <row r="549">
       <c r="A549" s="21" t="str">
-        <f>data!$B$77</f>
+        <f>data!$B$75</f>
       </c>
       <c r="B549" s="21"/>
       <c r="C549" s="21"/>
@@ -16328,10 +16328,10 @@
       <c r="E549" s="21"/>
       <c r="F549" s="21"/>
       <c r="G549" s="21" t="str">
-        <f>data!$B$76</f>
+        <f>data!$B$77</f>
       </c>
       <c r="I549" s="21" t="str">
-        <f>data!$B$80</f>
+        <f>data!$B$78</f>
       </c>
       <c r="J549" s="21"/>
       <c r="K549" s="21"/>
@@ -16339,7 +16339,7 @@
       <c r="M549" s="21"/>
       <c r="N549" s="21"/>
       <c r="O549" s="21" t="str">
-        <f>data!$B$79</f>
+        <f>data!$B$80</f>
       </c>
     </row>
     <row r="550">
@@ -16464,7 +16464,7 @@
     </row>
     <row r="556">
       <c r="A556" s="21" t="str">
-        <f>data!$B$77</f>
+        <f>data!$B$75</f>
       </c>
       <c r="B556" s="21" t="s">
         <v>239</v>
@@ -16480,10 +16480,10 @@
         <v>239</v>
       </c>
       <c r="G556" s="21" t="str">
-        <f>data!$B$76</f>
+        <f>data!$B$77</f>
       </c>
       <c r="I556" s="21" t="str">
-        <f>data!$B$80</f>
+        <f>data!$B$78</f>
       </c>
       <c r="J556" s="21" t="s">
         <v>239</v>
@@ -16499,7 +16499,7 @@
         <v>239</v>
       </c>
       <c r="O556" s="21" t="str">
-        <f>data!$B$79</f>
+        <f>data!$B$80</f>
       </c>
     </row>
     <row r="557">
@@ -16556,7 +16556,7 @@
     </row>
     <row r="562">
       <c r="A562" s="21" t="str">
-        <f>data!$B$77</f>
+        <f>data!$B$76</f>
       </c>
       <c r="B562" s="21"/>
       <c r="C562" s="21"/>
@@ -16564,10 +16564,10 @@
       <c r="E562" s="21"/>
       <c r="F562" s="21"/>
       <c r="G562" s="21" t="str">
-        <f>data!$B$75</f>
+        <f>data!$B$77</f>
       </c>
       <c r="I562" s="21" t="str">
-        <f>data!$B$80</f>
+        <f>data!$B$79</f>
       </c>
       <c r="J562" s="21"/>
       <c r="K562" s="21"/>
@@ -16575,7 +16575,7 @@
       <c r="M562" s="21"/>
       <c r="N562" s="21"/>
       <c r="O562" s="21" t="str">
-        <f>data!$B$78</f>
+        <f>data!$B$80</f>
       </c>
     </row>
     <row r="563">
@@ -16700,7 +16700,7 @@
     </row>
     <row r="569">
       <c r="A569" s="21" t="str">
-        <f>data!$B$77</f>
+        <f>data!$B$76</f>
       </c>
       <c r="B569" s="21" t="s">
         <v>239</v>
@@ -16716,10 +16716,10 @@
         <v>239</v>
       </c>
       <c r="G569" s="21" t="str">
-        <f>data!$B$75</f>
+        <f>data!$B$77</f>
       </c>
       <c r="I569" s="21" t="str">
-        <f>data!$B$80</f>
+        <f>data!$B$79</f>
       </c>
       <c r="J569" s="21" t="s">
         <v>239</v>
@@ -16735,7 +16735,7 @@
         <v>239</v>
       </c>
       <c r="O569" s="21" t="str">
-        <f>data!$B$78</f>
+        <f>data!$B$80</f>
       </c>
     </row>
     <row r="570">
@@ -17078,7 +17078,7 @@
     </row>
     <row r="592">
       <c r="A592" s="21" t="str">
-        <f>data!$B$83</f>
+        <f>data!$B$81</f>
       </c>
       <c r="B592" s="21"/>
       <c r="C592" s="21"/>
@@ -17086,10 +17086,10 @@
       <c r="E592" s="21"/>
       <c r="F592" s="21"/>
       <c r="G592" s="21" t="str">
-        <f>data!$B$82</f>
+        <f>data!$B$83</f>
       </c>
       <c r="I592" s="21" t="str">
-        <f>data!$B$86</f>
+        <f>data!$B$84</f>
       </c>
       <c r="J592" s="21"/>
       <c r="K592" s="21"/>
@@ -17097,7 +17097,7 @@
       <c r="M592" s="21"/>
       <c r="N592" s="21"/>
       <c r="O592" s="21" t="str">
-        <f>data!$B$85</f>
+        <f>data!$B$86</f>
       </c>
     </row>
     <row r="593">
@@ -17222,7 +17222,7 @@
     </row>
     <row r="599">
       <c r="A599" s="21" t="str">
-        <f>data!$B$83</f>
+        <f>data!$B$81</f>
       </c>
       <c r="B599" s="21" t="s">
         <v>239</v>
@@ -17238,10 +17238,10 @@
         <v>239</v>
       </c>
       <c r="G599" s="21" t="str">
-        <f>data!$B$82</f>
+        <f>data!$B$83</f>
       </c>
       <c r="I599" s="21" t="str">
-        <f>data!$B$86</f>
+        <f>data!$B$84</f>
       </c>
       <c r="J599" s="21" t="s">
         <v>239</v>
@@ -17257,7 +17257,7 @@
         <v>239</v>
       </c>
       <c r="O599" s="21" t="str">
-        <f>data!$B$85</f>
+        <f>data!$B$86</f>
       </c>
     </row>
     <row r="600">
@@ -17314,7 +17314,7 @@
     </row>
     <row r="605">
       <c r="A605" s="21" t="str">
-        <f>data!$B$83</f>
+        <f>data!$B$82</f>
       </c>
       <c r="B605" s="21"/>
       <c r="C605" s="21"/>
@@ -17322,10 +17322,10 @@
       <c r="E605" s="21"/>
       <c r="F605" s="21"/>
       <c r="G605" s="21" t="str">
-        <f>data!$B$81</f>
+        <f>data!$B$83</f>
       </c>
       <c r="I605" s="21" t="str">
-        <f>data!$B$86</f>
+        <f>data!$B$85</f>
       </c>
       <c r="J605" s="21"/>
       <c r="K605" s="21"/>
@@ -17333,7 +17333,7 @@
       <c r="M605" s="21"/>
       <c r="N605" s="21"/>
       <c r="O605" s="21" t="str">
-        <f>data!$B$84</f>
+        <f>data!$B$86</f>
       </c>
     </row>
     <row r="606">
@@ -17458,7 +17458,7 @@
     </row>
     <row r="612">
       <c r="A612" s="21" t="str">
-        <f>data!$B$83</f>
+        <f>data!$B$82</f>
       </c>
       <c r="B612" s="21" t="s">
         <v>239</v>
@@ -17474,10 +17474,10 @@
         <v>239</v>
       </c>
       <c r="G612" s="21" t="str">
-        <f>data!$B$81</f>
+        <f>data!$B$83</f>
       </c>
       <c r="I612" s="21" t="str">
-        <f>data!$B$86</f>
+        <f>data!$B$85</f>
       </c>
       <c r="J612" s="21" t="s">
         <v>239</v>
@@ -17493,7 +17493,7 @@
         <v>239</v>
       </c>
       <c r="O612" s="21" t="str">
-        <f>data!$B$84</f>
+        <f>data!$B$86</f>
       </c>
     </row>
     <row r="613">
@@ -17836,7 +17836,7 @@
     </row>
     <row r="635">
       <c r="A635" s="21" t="str">
-        <f>data!$B$89</f>
+        <f>data!$B$87</f>
       </c>
       <c r="B635" s="21"/>
       <c r="C635" s="21"/>
@@ -17844,10 +17844,10 @@
       <c r="E635" s="21"/>
       <c r="F635" s="21"/>
       <c r="G635" s="21" t="str">
-        <f>data!$B$88</f>
+        <f>data!$B$89</f>
       </c>
       <c r="I635" s="21" t="str">
-        <f>data!$B$92</f>
+        <f>data!$B$90</f>
       </c>
       <c r="J635" s="21"/>
       <c r="K635" s="21"/>
@@ -17855,7 +17855,7 @@
       <c r="M635" s="21"/>
       <c r="N635" s="21"/>
       <c r="O635" s="21" t="str">
-        <f>data!$B$91</f>
+        <f>data!$B$92</f>
       </c>
     </row>
     <row r="636">
@@ -17980,7 +17980,7 @@
     </row>
     <row r="642">
       <c r="A642" s="21" t="str">
-        <f>data!$B$89</f>
+        <f>data!$B$87</f>
       </c>
       <c r="B642" s="21" t="s">
         <v>239</v>
@@ -17996,10 +17996,10 @@
         <v>239</v>
       </c>
       <c r="G642" s="21" t="str">
-        <f>data!$B$88</f>
+        <f>data!$B$89</f>
       </c>
       <c r="I642" s="21" t="str">
-        <f>data!$B$92</f>
+        <f>data!$B$90</f>
       </c>
       <c r="J642" s="21" t="s">
         <v>239</v>
@@ -18015,7 +18015,7 @@
         <v>239</v>
       </c>
       <c r="O642" s="21" t="str">
-        <f>data!$B$91</f>
+        <f>data!$B$92</f>
       </c>
     </row>
     <row r="643">
@@ -18072,7 +18072,7 @@
     </row>
     <row r="648">
       <c r="A648" s="21" t="str">
-        <f>data!$B$89</f>
+        <f>data!$B$88</f>
       </c>
       <c r="B648" s="21"/>
       <c r="C648" s="21"/>
@@ -18080,10 +18080,10 @@
       <c r="E648" s="21"/>
       <c r="F648" s="21"/>
       <c r="G648" s="21" t="str">
-        <f>data!$B$87</f>
+        <f>data!$B$89</f>
       </c>
       <c r="I648" s="21" t="str">
-        <f>data!$B$92</f>
+        <f>data!$B$91</f>
       </c>
       <c r="J648" s="21"/>
       <c r="K648" s="21"/>
@@ -18091,7 +18091,7 @@
       <c r="M648" s="21"/>
       <c r="N648" s="21"/>
       <c r="O648" s="21" t="str">
-        <f>data!$B$90</f>
+        <f>data!$B$92</f>
       </c>
     </row>
     <row r="649">
@@ -18216,7 +18216,7 @@
     </row>
     <row r="655">
       <c r="A655" s="21" t="str">
-        <f>data!$B$89</f>
+        <f>data!$B$88</f>
       </c>
       <c r="B655" s="21" t="s">
         <v>239</v>
@@ -18232,10 +18232,10 @@
         <v>239</v>
       </c>
       <c r="G655" s="21" t="str">
-        <f>data!$B$87</f>
+        <f>data!$B$89</f>
       </c>
       <c r="I655" s="21" t="str">
-        <f>data!$B$92</f>
+        <f>data!$B$91</f>
       </c>
       <c r="J655" s="21" t="s">
         <v>239</v>
@@ -18251,7 +18251,7 @@
         <v>239</v>
       </c>
       <c r="O655" s="21" t="str">
-        <f>data!$B$90</f>
+        <f>data!$B$92</f>
       </c>
     </row>
     <row r="656">

</xml_diff>